<commit_message>
added chmod tests + helper functions
</commit_message>
<xml_diff>
--- a/individual_Tests/read/read_test_results.xlsx
+++ b/individual_Tests/read/read_test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Masters\Tests\initial_tests\individual_Tests\read\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8478568-4BC4-46EA-9407-85821E0F9986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DFC4744-2185-4D24-B708-907201261253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -220,10 +220,10 @@
     <t xml:space="preserve">Similar to write_03, basically read does not respect permissions since there is no check of the permissions of the fd in the syscal (O_ACCMODE).  </t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Patched?</t>
+  </si>
+  <si>
+    <t>Yes, 1db8e2d</t>
   </si>
 </sst>
 </file>
@@ -368,11 +368,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -691,17 +691,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -729,7 +729,7 @@
         <v>7</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -805,8 +805,8 @@
       <c r="H5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="I5" s="11" t="s">
-        <v>65</v>
+      <c r="I5" s="12" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KLEE test suite: added chmod tests + helper functions
</commit_message>
<xml_diff>
--- a/individual_Tests/read/read_test_results.xlsx
+++ b/individual_Tests/read/read_test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Masters\Tests\initial_tests\individual_Tests\read\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8478568-4BC4-46EA-9407-85821E0F9986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DFC4744-2185-4D24-B708-907201261253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -220,10 +220,10 @@
     <t xml:space="preserve">Similar to write_03, basically read does not respect permissions since there is no check of the permissions of the fd in the syscal (O_ACCMODE).  </t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Patched?</t>
+  </si>
+  <si>
+    <t>Yes, 1db8e2d</t>
   </si>
 </sst>
 </file>
@@ -368,11 +368,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -691,17 +691,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -729,7 +729,7 @@
         <v>7</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -805,8 +805,8 @@
       <c r="H5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="I5" s="11" t="s">
-        <v>65</v>
+      <c r="I5" s="12" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>